<commit_message>
Données mises à jour: +2 objets (Fridez inclus), total 142
</commit_message>
<xml_diff>
--- a/Nouveautés/Nouveautes_2026-03-26.xlsx
+++ b/Nouveautés/Nouveautes_2026-03-26.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t xml:space="preserve">Type_Changement</t>
   </si>
@@ -35,121 +35,28 @@
     <t xml:space="preserve">Nouvel objet</t>
   </si>
   <si>
-    <t xml:space="preserve">25.467</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stettler Thomas</t>
+    <t xml:space="preserve">25.4531</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fridez Pierre-Alain</t>
   </si>
   <si>
     <t xml:space="preserve">Titre uniquement</t>
   </si>
   <si>
-    <t xml:space="preserve">Vorprüfung - in Kommission des Nationalrates / Examen préalable - en commission du Conseil national</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20250467</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.4317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dobler Marcel</t>
-  </si>
-  <si>
     <t xml:space="preserve">Stellungnahme zum Vorstoss liegt vor / L’avis relatif à l’intervention est disponible</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.4380</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crevoisier Crelier Mathilde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zugewiesen an die behandelnde Kommission / Attribué à la commission compétente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254380</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.4686</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juillard Charles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254686</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.4687</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Überwiesen an den Bundesrat / Transmis au Conseil fédéral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254687</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.4774</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254774</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.4794</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254794</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.7664</t>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20254531</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26.7194</t>
   </si>
   <si>
     <t xml:space="preserve">Erledigt / Liquidé</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20257664</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25.8270</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20258270</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3099</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eingereicht / Déposé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263099</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3121</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263121</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3411</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263411</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.3454</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20263454</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.7185</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267185</t>
+    <t xml:space="preserve">https://www.parlament.ch/fr/ratsbetrieb/suche-curia-vista/geschaeft?AffairId=20267194</t>
   </si>
 </sst>
 </file>
@@ -197,8 +104,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:F15" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:F3" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:F3"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Type_Changement"/>
     <tableColumn id="2" name="Numéro"/>
@@ -541,256 +448,16 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
         <v>9</v>
       </c>
       <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
         <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" t="s">
-        <v>36</v>
-      </c>
-      <c r="F13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" t="s">
-        <v>36</v>
-      </c>
-      <c r="F14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" t="s">
-        <v>31</v>
-      </c>
-      <c r="F15" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>